<commit_message>
fix(internacional): lo opcional del resumen de unidad de HK S1–3 no es núcleo
corregir-metadatos marca como especialización lo que un documento con
Extension Part presenta como sugerencia al docente («Teachers may further
guide…»). Afecta un objetivo (HK-FIS-hk_s1_3-p062-22, gases); ninguna clase
final cambia. Singapur K326–K328 queda verificado (p. 6, «two of Papers 2, 3
and 4») y pendiente de decisión, con recomendación, en panel/bucle/README.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/2_8/Contraste_fisica.xlsx
+++ b/internacional/2_8/Contraste_fisica.xlsx
@@ -5424,9 +5424,6 @@
       <c r="G69" t="n">
         <v>8.5</v>
       </c>
-      <c r="H69" t="n">
-        <v>7</v>
-      </c>
       <c r="I69" t="n">
         <v>3</v>
       </c>
@@ -5439,9 +5436,6 @@
       <c r="P69" t="n">
         <v>1</v>
       </c>
-      <c r="Q69" t="n">
-        <v>1</v>
-      </c>
       <c r="R69" t="n">
         <v>1</v>
       </c>
@@ -5464,7 +5458,7 @@
       </c>
       <c r="AH69" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>posterior</t>
         </is>
       </c>
     </row>
@@ -7424,9 +7418,6 @@
       <c r="G110" t="n">
         <v>6</v>
       </c>
-      <c r="H110" t="n">
-        <v>7</v>
-      </c>
       <c r="J110" t="n">
         <v>2.5</v>
       </c>
@@ -7436,13 +7427,13 @@
       <c r="P110" t="n">
         <v>1</v>
       </c>
-      <c r="Q110" t="n">
-        <v>1</v>
-      </c>
       <c r="S110" t="n">
         <v>1</v>
       </c>
       <c r="V110" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z110" t="n">
         <v>1</v>
       </c>
       <c r="AF110" t="n">

</xml_diff>